<commit_message>
Add module detection for incompatible and cheat modules
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/src/other/gfx_addresses.xlsx
+++ b/src/other/gfx_addresses.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CoD2x\src\other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B6E42C-E614-4A1D-B23B-C10354EEA575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAEB304F-19C3-40F8-924C-7CDAB3A9F71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{52A9D2E3-6951-4E66-B218-1C49B54338DB}"/>
+    <workbookView xWindow="38280" yWindow="-5685" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{52A9D2E3-6951-4E66-B218-1C49B54338DB}"/>
   </bookViews>
   <sheets>
     <sheet name="CoD2 -&gt; Renderer" sheetId="3" r:id="rId1"/>
@@ -2538,9 +2538,6 @@
     <t>&amp;data_10020f90</t>
   </si>
   <si>
-    <t>sub_10013040</t>
-  </si>
-  <si>
     <t>R_DefaultVertexFrames</t>
   </si>
   <si>
@@ -3162,9 +3159,6 @@
     <t xml:space="preserve">void*&amp; data_10020f90 </t>
   </si>
   <si>
-    <t xml:space="preserve">void* sub_10013040 </t>
-  </si>
-  <si>
     <t xml:space="preserve">void* R_DefaultVertexFrames </t>
   </si>
   <si>
@@ -3736,6 +3730,12 @@
   </si>
   <si>
     <t>int32_t R_CreateRenderThread</t>
+  </si>
+  <si>
+    <t>void* createRenderThread</t>
+  </si>
+  <si>
+    <t>createRenderThread</t>
   </si>
 </sst>
 </file>
@@ -4348,13 +4348,13 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1102</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>1103</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>1104</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>1105</v>
       </c>
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
@@ -7332,7 +7332,7 @@
         <v>464</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
       <c r="D118" s="4" t="s">
         <v>506</v>
@@ -7344,7 +7344,7 @@
         <v>379</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="119" spans="2:10" x14ac:dyDescent="0.25">
@@ -7432,7 +7432,7 @@
         <v>484</v>
       </c>
       <c r="C123" s="6" t="s">
-        <v>1229</v>
+        <v>1227</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>506</v>
@@ -8792,16 +8792,16 @@
   <sheetData>
     <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="K1" s="1" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="L1" s="24" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.25">
@@ -8809,13 +8809,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="22" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F2" s="2" t="str">
         <f>DEC2HEX(G2)</f>
@@ -8831,17 +8831,17 @@
         <v>796</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="L2" s="24">
         <v>0</v>
       </c>
       <c r="M2" s="1">
-        <f>HEX2DEC(L2)</f>
+        <f t="shared" ref="M2:M20" si="0">HEX2DEC(L2)</f>
         <v>0</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>1219</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="3" spans="2:14" x14ac:dyDescent="0.25">
@@ -8849,16 +8849,16 @@
         <v>4</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F3" s="5" t="str">
-        <f t="shared" ref="F3:F66" si="0">DEC2HEX(G3)</f>
+        <f t="shared" ref="F3:F66" si="1">DEC2HEX(G3)</f>
         <v>1</v>
       </c>
       <c r="G3" s="9">
@@ -8871,13 +8871,13 @@
         <v>797</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="L3" s="24">
         <v>1</v>
       </c>
       <c r="M3" s="1">
-        <f>HEX2DEC(L3)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="N3" s="1" t="s">
@@ -8889,16 +8889,16 @@
         <v>8</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F4" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="G4" s="9">
@@ -8911,13 +8911,13 @@
         <v>798</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="L4" s="24">
         <v>2</v>
       </c>
       <c r="M4" s="1">
-        <f>HEX2DEC(L4)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="N4" s="1" t="s">
@@ -8929,16 +8929,16 @@
         <v>12</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F5" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="G5" s="9">
@@ -8951,13 +8951,13 @@
         <v>799</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="L5" s="24">
         <v>3</v>
       </c>
       <c r="M5" s="1">
-        <f>HEX2DEC(L5)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="N5" s="1" t="s">
@@ -8969,16 +8969,16 @@
         <v>16</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F6" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="G6" s="9">
@@ -8991,13 +8991,13 @@
         <v>801</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="L6" s="24">
         <v>4</v>
       </c>
       <c r="M6" s="1">
-        <f>HEX2DEC(L6)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="N6" s="1" t="s">
@@ -9009,16 +9009,16 @@
         <v>20</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F7" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="G7" s="9">
@@ -9031,13 +9031,13 @@
         <v>802</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="L7" s="24">
         <v>5</v>
       </c>
       <c r="M7" s="1">
-        <f>HEX2DEC(L7)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -9049,16 +9049,16 @@
         <v>24</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F8" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="G8" s="9">
@@ -9071,13 +9071,13 @@
         <v>803</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="L8" s="24">
         <v>6</v>
       </c>
       <c r="M8" s="1">
-        <f>HEX2DEC(L8)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="N8" s="1" t="s">
@@ -9089,16 +9089,16 @@
         <v>28</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F9" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="G9" s="9">
@@ -9111,13 +9111,13 @@
         <v>804</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="L9" s="24">
         <v>7</v>
       </c>
       <c r="M9" s="1">
-        <f>HEX2DEC(L9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="N9" s="1" t="s">
@@ -9129,16 +9129,16 @@
         <v>32</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F10" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="G10" s="9">
@@ -9151,13 +9151,13 @@
         <v>805</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="L10" s="24">
         <v>8</v>
       </c>
       <c r="M10" s="1">
-        <f>HEX2DEC(L10)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="N10" s="1" t="s">
@@ -9169,16 +9169,16 @@
         <v>36</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F11" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="G11" s="9">
@@ -9191,13 +9191,13 @@
         <v>806</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="L11" s="24">
         <v>9</v>
       </c>
       <c r="M11" s="1">
-        <f>HEX2DEC(L11)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="N11" s="1" t="s">
@@ -9209,16 +9209,16 @@
         <v>40</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F12" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>A</v>
       </c>
       <c r="G12" s="9">
@@ -9231,13 +9231,13 @@
         <v>807</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="L12" s="24" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="M12" s="1">
-        <f>HEX2DEC(L12)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="N12" s="1" t="s">
@@ -9249,16 +9249,16 @@
         <v>44</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F13" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>B</v>
       </c>
       <c r="G13" s="9">
@@ -9271,13 +9271,13 @@
         <v>808</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="L13" s="24" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="M13" s="1">
-        <f>HEX2DEC(L13)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="N13" s="1" t="s">
@@ -9289,16 +9289,16 @@
         <v>48</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F14" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>C</v>
       </c>
       <c r="G14" s="9">
@@ -9311,13 +9311,13 @@
         <v>800</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="L14" s="24" t="s">
         <v>146</v>
       </c>
       <c r="M14" s="1">
-        <f>HEX2DEC(L14)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="N14" s="1" t="s">
@@ -9329,16 +9329,16 @@
         <v>52</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F15" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>D</v>
       </c>
       <c r="G15" s="9">
@@ -9351,13 +9351,13 @@
         <v>810</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="L15" s="24" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="M15" s="1">
-        <f>HEX2DEC(L15)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="N15" s="1" t="s">
@@ -9369,16 +9369,16 @@
         <v>56</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F16" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>E</v>
       </c>
       <c r="G16" s="9">
@@ -9391,13 +9391,13 @@
         <v>811</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="L16" s="24" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="M16" s="1">
-        <f>HEX2DEC(L16)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="N16" s="1" t="s">
@@ -9409,16 +9409,16 @@
         <v>60</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F17" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>F</v>
       </c>
       <c r="G17" s="9">
@@ -9431,13 +9431,13 @@
         <v>812</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="L17" s="24" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="M17" s="1">
-        <f>HEX2DEC(L17)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="N17" s="1" t="s">
@@ -9449,16 +9449,16 @@
         <v>64</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F18" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="G18" s="9">
@@ -9471,13 +9471,13 @@
         <v>813</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="L18" s="24">
         <v>10</v>
       </c>
       <c r="M18" s="1">
-        <f>HEX2DEC(L18)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="N18" s="1" t="s">
@@ -9489,16 +9489,16 @@
         <v>68</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F19" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="G19" s="9">
@@ -9511,13 +9511,13 @@
         <v>809</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="L19" s="24">
         <v>11</v>
       </c>
       <c r="M19" s="1">
-        <f>HEX2DEC(L19)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="N19" s="1" t="s">
@@ -9529,16 +9529,16 @@
         <v>72</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F20" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="G20" s="9">
@@ -9551,13 +9551,13 @@
         <v>826</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="L20" s="24">
         <v>12</v>
       </c>
       <c r="M20" s="1">
-        <f>HEX2DEC(L20)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="N20" s="1" t="s">
@@ -9569,16 +9569,16 @@
         <v>76</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F21" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
       <c r="G21" s="9">
@@ -9596,16 +9596,16 @@
         <v>80</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F22" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="G22" s="9">
@@ -9623,16 +9623,16 @@
         <v>84</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F23" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="G23" s="9">
@@ -9650,16 +9650,16 @@
         <v>88</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F24" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="G24" s="9">
@@ -9677,16 +9677,16 @@
         <v>92</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F25" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="G25" s="9">
@@ -9704,16 +9704,16 @@
         <v>96</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1040</v>
+        <v>1230</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F26" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="G26" s="9">
@@ -9723,7 +9723,7 @@
         <v>96</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>832</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
@@ -9731,16 +9731,16 @@
         <v>100</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F27" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
       <c r="G27" s="9">
@@ -9750,20 +9750,20 @@
         <v>100</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="L27" s="24">
         <v>13</v>
       </c>
       <c r="M27" s="1">
-        <f>HEX2DEC(L27)</f>
+        <f t="shared" ref="M27:M58" si="2">HEX2DEC(L27)</f>
         <v>19</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
@@ -9771,16 +9771,16 @@
         <v>104</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F28" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1A</v>
       </c>
       <c r="G28" s="9">
@@ -9790,20 +9790,20 @@
         <v>104</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="L28" s="24">
         <v>14</v>
       </c>
       <c r="M28" s="1">
-        <f>HEX2DEC(L28)</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
@@ -9811,16 +9811,16 @@
         <v>108</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F29" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1B</v>
       </c>
       <c r="G29" s="9">
@@ -9830,20 +9830,20 @@
         <v>108</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="L29" s="24">
         <v>15</v>
       </c>
       <c r="M29" s="1">
-        <f>HEX2DEC(L29)</f>
+        <f t="shared" si="2"/>
         <v>21</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
@@ -9851,16 +9851,16 @@
         <v>112</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F30" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1C</v>
       </c>
       <c r="G30" s="9">
@@ -9870,20 +9870,20 @@
         <v>112</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="L30" s="24">
         <v>16</v>
       </c>
       <c r="M30" s="1">
-        <f>HEX2DEC(L30)</f>
+        <f t="shared" si="2"/>
         <v>22</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
@@ -9891,16 +9891,16 @@
         <v>116</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F31" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1D</v>
       </c>
       <c r="G31" s="9">
@@ -9910,20 +9910,20 @@
         <v>116</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="L31" s="24">
         <v>17</v>
       </c>
       <c r="M31" s="1">
-        <f>HEX2DEC(L31)</f>
+        <f t="shared" si="2"/>
         <v>23</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
@@ -9931,16 +9931,16 @@
         <v>120</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F32" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1E</v>
       </c>
       <c r="G32" s="9">
@@ -9950,20 +9950,20 @@
         <v>120</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="L32" s="24">
         <v>18</v>
       </c>
       <c r="M32" s="1">
-        <f>HEX2DEC(L32)</f>
+        <f t="shared" si="2"/>
         <v>24</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
@@ -9971,16 +9971,16 @@
         <v>124</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F33" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1F</v>
       </c>
       <c r="G33" s="9">
@@ -9990,20 +9990,20 @@
         <v>124</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="L33" s="24">
         <v>19</v>
       </c>
       <c r="M33" s="1">
-        <f>HEX2DEC(L33)</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
@@ -10011,16 +10011,16 @@
         <v>128</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F34" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="G34" s="9">
@@ -10030,20 +10030,20 @@
         <v>128</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="L34" s="24" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="M34" s="1">
-        <f>HEX2DEC(L34)</f>
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
@@ -10051,16 +10051,16 @@
         <v>132</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F35" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="G35" s="9">
@@ -10070,20 +10070,20 @@
         <v>132</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="L35" s="24" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="M35" s="1">
-        <f>HEX2DEC(L35)</f>
+        <f t="shared" si="2"/>
         <v>27</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
@@ -10091,16 +10091,16 @@
         <v>136</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F36" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="G36" s="9">
@@ -10110,20 +10110,20 @@
         <v>136</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="L36" s="24" t="s">
         <v>147</v>
       </c>
       <c r="M36" s="1">
-        <f>HEX2DEC(L36)</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
@@ -10131,16 +10131,16 @@
         <v>140</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F37" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="G37" s="9">
@@ -10150,20 +10150,20 @@
         <v>140</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="L37" s="24" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="M37" s="1">
-        <f>HEX2DEC(L37)</f>
+        <f t="shared" si="2"/>
         <v>29</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
@@ -10171,16 +10171,16 @@
         <v>144</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F38" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="G38" s="9">
@@ -10190,20 +10190,20 @@
         <v>144</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="L38" s="24" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="M38" s="1">
-        <f>HEX2DEC(L38)</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
@@ -10211,16 +10211,16 @@
         <v>148</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F39" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="G39" s="9">
@@ -10230,20 +10230,20 @@
         <v>148</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="L39" s="24" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="M39" s="1">
-        <f>HEX2DEC(L39)</f>
+        <f t="shared" si="2"/>
         <v>31</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
@@ -10251,16 +10251,16 @@
         <v>152</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F40" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="G40" s="9">
@@ -10270,20 +10270,20 @@
         <v>152</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="L40" s="24">
         <v>20</v>
       </c>
       <c r="M40" s="1">
-        <f>HEX2DEC(L40)</f>
+        <f t="shared" si="2"/>
         <v>32</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
@@ -10291,16 +10291,16 @@
         <v>156</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F41" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="G41" s="9">
@@ -10310,20 +10310,20 @@
         <v>156</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="L41" s="24">
         <v>21</v>
       </c>
       <c r="M41" s="1">
-        <f>HEX2DEC(L41)</f>
+        <f t="shared" si="2"/>
         <v>33</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
@@ -10331,16 +10331,16 @@
         <v>160</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F42" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="G42" s="9">
@@ -10350,20 +10350,20 @@
         <v>160</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="L42" s="24">
         <v>22</v>
       </c>
       <c r="M42" s="1">
-        <f>HEX2DEC(L42)</f>
+        <f t="shared" si="2"/>
         <v>34</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
@@ -10371,16 +10371,16 @@
         <v>164</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F43" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="G43" s="9">
@@ -10390,20 +10390,20 @@
         <v>164</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="L43" s="24">
         <v>23</v>
       </c>
       <c r="M43" s="1">
-        <f>HEX2DEC(L43)</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
@@ -10411,16 +10411,16 @@
         <v>168</v>
       </c>
       <c r="C44" s="21" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F44" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2A</v>
       </c>
       <c r="G44" s="9">
@@ -10430,20 +10430,20 @@
         <v>168</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="L44" s="24">
         <v>24</v>
       </c>
       <c r="M44" s="1">
-        <f>HEX2DEC(L44)</f>
+        <f t="shared" si="2"/>
         <v>36</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
@@ -10451,16 +10451,16 @@
         <v>172</v>
       </c>
       <c r="C45" s="21" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F45" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2B</v>
       </c>
       <c r="G45" s="9">
@@ -10470,20 +10470,20 @@
         <v>172</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="L45" s="24">
         <v>25</v>
       </c>
       <c r="M45" s="1">
-        <f>HEX2DEC(L45)</f>
+        <f t="shared" si="2"/>
         <v>37</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
@@ -10491,16 +10491,16 @@
         <v>176</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F46" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2C</v>
       </c>
       <c r="G46" s="9">
@@ -10510,20 +10510,20 @@
         <v>176</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="L46" s="24">
         <v>26</v>
       </c>
       <c r="M46" s="1">
-        <f>HEX2DEC(L46)</f>
+        <f t="shared" si="2"/>
         <v>38</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
@@ -10531,16 +10531,16 @@
         <v>180</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F47" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2D</v>
       </c>
       <c r="G47" s="9">
@@ -10550,20 +10550,20 @@
         <v>180</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="L47" s="24">
         <v>27</v>
       </c>
       <c r="M47" s="1">
-        <f>HEX2DEC(L47)</f>
+        <f t="shared" si="2"/>
         <v>39</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
@@ -10571,16 +10571,16 @@
         <v>184</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F48" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2E</v>
       </c>
       <c r="G48" s="9">
@@ -10590,20 +10590,20 @@
         <v>184</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="L48" s="24">
         <v>28</v>
       </c>
       <c r="M48" s="1">
-        <f>HEX2DEC(L48)</f>
+        <f t="shared" si="2"/>
         <v>40</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
@@ -10611,16 +10611,16 @@
         <v>188</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F49" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2F</v>
       </c>
       <c r="G49" s="9">
@@ -10630,20 +10630,20 @@
         <v>188</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="L49" s="24">
         <v>29</v>
       </c>
       <c r="M49" s="1">
-        <f>HEX2DEC(L49)</f>
+        <f t="shared" si="2"/>
         <v>41</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.25">
@@ -10651,16 +10651,16 @@
         <v>192</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F50" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="G50" s="9">
@@ -10673,13 +10673,13 @@
         <v>814</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="L50" s="24" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="M50" s="1">
-        <f>HEX2DEC(L50)</f>
+        <f t="shared" si="2"/>
         <v>42</v>
       </c>
       <c r="N50" s="1" t="s">
@@ -10691,16 +10691,16 @@
         <v>196</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F51" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="G51" s="9">
@@ -10713,13 +10713,13 @@
         <v>815</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="L51" s="24" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="M51" s="1">
-        <f>HEX2DEC(L51)</f>
+        <f t="shared" si="2"/>
         <v>43</v>
       </c>
       <c r="N51" s="1" t="s">
@@ -10731,16 +10731,16 @@
         <v>200</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F52" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>32</v>
       </c>
       <c r="G52" s="9">
@@ -10753,13 +10753,13 @@
         <v>816</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="L52" s="24" t="s">
         <v>148</v>
       </c>
       <c r="M52" s="1">
-        <f>HEX2DEC(L52)</f>
+        <f t="shared" si="2"/>
         <v>44</v>
       </c>
       <c r="N52" s="1" t="s">
@@ -10771,16 +10771,16 @@
         <v>204</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F53" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="G53" s="9">
@@ -10793,13 +10793,13 @@
         <v>817</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="L53" s="24" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="M53" s="1">
-        <f>HEX2DEC(L53)</f>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="N53" s="1" t="s">
@@ -10811,16 +10811,16 @@
         <v>208</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F54" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="G54" s="9">
@@ -10833,13 +10833,13 @@
         <v>818</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="L54" s="24" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="M54" s="1">
-        <f>HEX2DEC(L54)</f>
+        <f t="shared" si="2"/>
         <v>46</v>
       </c>
       <c r="N54" s="1" t="s">
@@ -10851,16 +10851,16 @@
         <v>212</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F55" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="G55" s="9">
@@ -10873,13 +10873,13 @@
         <v>819</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="L55" s="24" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="M55" s="1">
-        <f>HEX2DEC(L55)</f>
+        <f t="shared" si="2"/>
         <v>47</v>
       </c>
       <c r="N55" s="1" t="s">
@@ -10891,16 +10891,16 @@
         <v>216</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F56" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="G56" s="9">
@@ -10913,13 +10913,13 @@
         <v>820</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="L56" s="24">
         <v>30</v>
       </c>
       <c r="M56" s="1">
-        <f>HEX2DEC(L56)</f>
+        <f t="shared" si="2"/>
         <v>48</v>
       </c>
       <c r="N56" s="1" t="s">
@@ -10931,16 +10931,16 @@
         <v>220</v>
       </c>
       <c r="C57" s="21" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F57" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="G57" s="9">
@@ -10953,13 +10953,13 @@
         <v>821</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="L57" s="24">
         <v>31</v>
       </c>
       <c r="M57" s="1">
-        <f>HEX2DEC(L57)</f>
+        <f t="shared" si="2"/>
         <v>49</v>
       </c>
       <c r="N57" s="1" t="s">
@@ -10971,16 +10971,16 @@
         <v>224</v>
       </c>
       <c r="C58" s="21" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F58" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="G58" s="9">
@@ -10993,13 +10993,13 @@
         <v>822</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="L58" s="24">
         <v>32</v>
       </c>
       <c r="M58" s="1">
-        <f>HEX2DEC(L58)</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="N58" s="1" t="s">
@@ -11011,16 +11011,16 @@
         <v>228</v>
       </c>
       <c r="C59" s="21" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F59" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="G59" s="9">
@@ -11033,13 +11033,13 @@
         <v>823</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="L59" s="24">
         <v>33</v>
       </c>
       <c r="M59" s="1">
-        <f>HEX2DEC(L59)</f>
+        <f t="shared" ref="M59:M90" si="3">HEX2DEC(L59)</f>
         <v>51</v>
       </c>
       <c r="N59" s="1" t="s">
@@ -11051,16 +11051,16 @@
         <v>232</v>
       </c>
       <c r="C60" s="21" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F60" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3A</v>
       </c>
       <c r="G60" s="9">
@@ -11073,13 +11073,13 @@
         <v>824</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="L60" s="24">
         <v>34</v>
       </c>
       <c r="M60" s="1">
-        <f>HEX2DEC(L60)</f>
+        <f t="shared" si="3"/>
         <v>52</v>
       </c>
       <c r="N60" s="1" t="s">
@@ -11091,16 +11091,16 @@
         <v>236</v>
       </c>
       <c r="C61" s="21" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F61" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3B</v>
       </c>
       <c r="G61" s="9">
@@ -11113,13 +11113,13 @@
         <v>825</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="L61" s="24">
         <v>35</v>
       </c>
       <c r="M61" s="1">
-        <f>HEX2DEC(L61)</f>
+        <f t="shared" si="3"/>
         <v>53</v>
       </c>
       <c r="N61" s="1" t="s">
@@ -11131,16 +11131,16 @@
         <v>240</v>
       </c>
       <c r="C62" s="21" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F62" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3C</v>
       </c>
       <c r="G62" s="9">
@@ -11150,20 +11150,20 @@
         <v>240</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="L62" s="24">
         <v>36</v>
       </c>
       <c r="M62" s="1">
-        <f>HEX2DEC(L62)</f>
+        <f t="shared" si="3"/>
         <v>54</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
@@ -11171,16 +11171,16 @@
         <v>244</v>
       </c>
       <c r="C63" s="21" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F63" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3D</v>
       </c>
       <c r="G63" s="9">
@@ -11190,20 +11190,20 @@
         <v>244</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="L63" s="24">
         <v>37</v>
       </c>
       <c r="M63" s="1">
-        <f>HEX2DEC(L63)</f>
+        <f t="shared" si="3"/>
         <v>55</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
@@ -11211,16 +11211,16 @@
         <v>248</v>
       </c>
       <c r="C64" s="21" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F64" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3E</v>
       </c>
       <c r="G64" s="9">
@@ -11230,20 +11230,20 @@
         <v>248</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="K64" s="1" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="L64" s="24">
         <v>38</v>
       </c>
       <c r="M64" s="1">
-        <f>HEX2DEC(L64)</f>
+        <f t="shared" si="3"/>
         <v>56</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.25">
@@ -11251,16 +11251,16 @@
         <v>252</v>
       </c>
       <c r="C65" s="21" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F65" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3F</v>
       </c>
       <c r="G65" s="9">
@@ -11270,20 +11270,20 @@
         <v>252</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="K65" s="1" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="L65" s="24">
         <v>39</v>
       </c>
       <c r="M65" s="1">
-        <f>HEX2DEC(L65)</f>
+        <f t="shared" si="3"/>
         <v>57</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.25">
@@ -11291,16 +11291,16 @@
         <v>256</v>
       </c>
       <c r="C66" s="21" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F66" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="G66" s="9">
@@ -11310,20 +11310,20 @@
         <v>256</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="K66" s="1" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="L66" s="24" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="M66" s="1">
-        <f>HEX2DEC(L66)</f>
+        <f t="shared" si="3"/>
         <v>58</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.25">
@@ -11331,16 +11331,16 @@
         <v>260</v>
       </c>
       <c r="C67" s="21" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F67" s="5" t="str">
-        <f t="shared" ref="F67:F109" si="1">DEC2HEX(G67)</f>
+        <f t="shared" ref="F67:F109" si="4">DEC2HEX(G67)</f>
         <v>41</v>
       </c>
       <c r="G67" s="9">
@@ -11350,20 +11350,20 @@
         <v>260</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="K67" s="1" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="L67" s="24" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="M67" s="1">
-        <f>HEX2DEC(L67)</f>
+        <f t="shared" si="3"/>
         <v>59</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.25">
@@ -11371,16 +11371,16 @@
         <v>264</v>
       </c>
       <c r="C68" s="21" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F68" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>42</v>
       </c>
       <c r="G68" s="9">
@@ -11390,20 +11390,20 @@
         <v>264</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="L68" s="24" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="M68" s="1">
-        <f>HEX2DEC(L68)</f>
+        <f t="shared" si="3"/>
         <v>60</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.25">
@@ -11411,16 +11411,16 @@
         <v>268</v>
       </c>
       <c r="C69" s="21" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F69" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>43</v>
       </c>
       <c r="G69" s="9">
@@ -11430,20 +11430,20 @@
         <v>268</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="L69" s="24" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="M69" s="1">
-        <f>HEX2DEC(L69)</f>
+        <f t="shared" si="3"/>
         <v>61</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.25">
@@ -11451,16 +11451,16 @@
         <v>272</v>
       </c>
       <c r="C70" s="21" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F70" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>44</v>
       </c>
       <c r="G70" s="9">
@@ -11470,20 +11470,20 @@
         <v>272</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="K70" s="1" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="L70" s="24" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="M70" s="1">
-        <f>HEX2DEC(L70)</f>
+        <f t="shared" si="3"/>
         <v>62</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.25">
@@ -11491,16 +11491,16 @@
         <v>276</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F71" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>45</v>
       </c>
       <c r="G71" s="9">
@@ -11510,20 +11510,20 @@
         <v>276</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="L71" s="24" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="M71" s="1">
-        <f>HEX2DEC(L71)</f>
+        <f t="shared" si="3"/>
         <v>63</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.25">
@@ -11531,16 +11531,16 @@
         <v>280</v>
       </c>
       <c r="C72" s="21" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F72" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>46</v>
       </c>
       <c r="G72" s="9">
@@ -11550,20 +11550,20 @@
         <v>280</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="K72" s="1" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="L72" s="24">
         <v>40</v>
       </c>
       <c r="M72" s="1">
-        <f>HEX2DEC(L72)</f>
+        <f t="shared" si="3"/>
         <v>64</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.25">
@@ -11571,16 +11571,16 @@
         <v>284</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F73" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>47</v>
       </c>
       <c r="G73" s="9">
@@ -11590,20 +11590,20 @@
         <v>284</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="K73" s="1" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="L73" s="24">
         <v>41</v>
       </c>
       <c r="M73" s="1">
-        <f>HEX2DEC(L73)</f>
+        <f t="shared" si="3"/>
         <v>65</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.25">
@@ -11611,16 +11611,16 @@
         <v>288</v>
       </c>
       <c r="C74" s="21" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F74" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>48</v>
       </c>
       <c r="G74" s="9">
@@ -11630,20 +11630,20 @@
         <v>288</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="L74" s="24">
         <v>42</v>
       </c>
       <c r="M74" s="1">
-        <f>HEX2DEC(L74)</f>
+        <f t="shared" si="3"/>
         <v>66</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.25">
@@ -11651,16 +11651,16 @@
         <v>292</v>
       </c>
       <c r="C75" s="21" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F75" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>49</v>
       </c>
       <c r="G75" s="9">
@@ -11670,20 +11670,20 @@
         <v>292</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="K75" s="1" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="L75" s="24">
         <v>43</v>
       </c>
       <c r="M75" s="1">
-        <f>HEX2DEC(L75)</f>
+        <f t="shared" si="3"/>
         <v>67</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.25">
@@ -11691,16 +11691,16 @@
         <v>296</v>
       </c>
       <c r="C76" s="21" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F76" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4A</v>
       </c>
       <c r="G76" s="9">
@@ -11710,20 +11710,20 @@
         <v>296</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="K76" s="1" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="L76" s="24">
         <v>44</v>
       </c>
       <c r="M76" s="1">
-        <f>HEX2DEC(L76)</f>
+        <f t="shared" si="3"/>
         <v>68</v>
       </c>
       <c r="N76" s="1" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.25">
@@ -11731,16 +11731,16 @@
         <v>300</v>
       </c>
       <c r="C77" s="21" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F77" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4B</v>
       </c>
       <c r="G77" s="9">
@@ -11750,20 +11750,20 @@
         <v>300</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="K77" s="1" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="L77" s="24">
         <v>45</v>
       </c>
       <c r="M77" s="1">
-        <f>HEX2DEC(L77)</f>
+        <f t="shared" si="3"/>
         <v>69</v>
       </c>
       <c r="N77" s="1" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.25">
@@ -11771,16 +11771,16 @@
         <v>304</v>
       </c>
       <c r="C78" s="21" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F78" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4C</v>
       </c>
       <c r="G78" s="9">
@@ -11790,20 +11790,20 @@
         <v>304</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="K78" s="1" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="L78" s="24">
         <v>46</v>
       </c>
       <c r="M78" s="1">
-        <f>HEX2DEC(L78)</f>
+        <f t="shared" si="3"/>
         <v>70</v>
       </c>
       <c r="N78" s="1" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.25">
@@ -11811,16 +11811,16 @@
         <v>308</v>
       </c>
       <c r="C79" s="21" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F79" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4D</v>
       </c>
       <c r="G79" s="9">
@@ -11830,20 +11830,20 @@
         <v>308</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="K79" s="1" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="L79" s="24">
         <v>47</v>
       </c>
       <c r="M79" s="1">
-        <f>HEX2DEC(L79)</f>
+        <f t="shared" si="3"/>
         <v>71</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.25">
@@ -11851,16 +11851,16 @@
         <v>312</v>
       </c>
       <c r="C80" s="21" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F80" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4E</v>
       </c>
       <c r="G80" s="9">
@@ -11870,20 +11870,20 @@
         <v>312</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="K80" s="1" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="L80" s="24">
         <v>48</v>
       </c>
       <c r="M80" s="1">
-        <f>HEX2DEC(L80)</f>
+        <f t="shared" si="3"/>
         <v>72</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.25">
@@ -11891,16 +11891,16 @@
         <v>316</v>
       </c>
       <c r="C81" s="21" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F81" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4F</v>
       </c>
       <c r="G81" s="9">
@@ -11910,20 +11910,20 @@
         <v>316</v>
       </c>
       <c r="I81" s="6" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="K81" s="1" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="L81" s="24">
         <v>49</v>
       </c>
       <c r="M81" s="1">
-        <f>HEX2DEC(L81)</f>
+        <f t="shared" si="3"/>
         <v>73</v>
       </c>
       <c r="N81" s="1" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.25">
@@ -11931,16 +11931,16 @@
         <v>320</v>
       </c>
       <c r="C82" s="21" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F82" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>50</v>
       </c>
       <c r="G82" s="9">
@@ -11950,20 +11950,20 @@
         <v>320</v>
       </c>
       <c r="I82" s="6" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="K82" s="1" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
       <c r="L82" s="24" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="M82" s="1">
-        <f>HEX2DEC(L82)</f>
+        <f t="shared" si="3"/>
         <v>74</v>
       </c>
       <c r="N82" s="1" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.25">
@@ -11971,16 +11971,16 @@
         <v>324</v>
       </c>
       <c r="C83" s="21" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F83" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>51</v>
       </c>
       <c r="G83" s="9">
@@ -11990,20 +11990,20 @@
         <v>324</v>
       </c>
       <c r="I83" s="6" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="L83" s="24" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="M83" s="1">
-        <f>HEX2DEC(L83)</f>
+        <f t="shared" si="3"/>
         <v>75</v>
       </c>
       <c r="N83" s="1" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.25">
@@ -12011,16 +12011,16 @@
         <v>328</v>
       </c>
       <c r="C84" s="21" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F84" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>52</v>
       </c>
       <c r="G84" s="9">
@@ -12030,20 +12030,20 @@
         <v>328</v>
       </c>
       <c r="I84" s="6" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="L84" s="24" t="s">
         <v>149</v>
       </c>
       <c r="M84" s="1">
-        <f>HEX2DEC(L84)</f>
+        <f t="shared" si="3"/>
         <v>76</v>
       </c>
       <c r="N84" s="1" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.25">
@@ -12051,16 +12051,16 @@
         <v>332</v>
       </c>
       <c r="C85" s="21" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F85" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>53</v>
       </c>
       <c r="G85" s="9">
@@ -12070,20 +12070,20 @@
         <v>332</v>
       </c>
       <c r="I85" s="6" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="K85" s="1" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="L85" s="24" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="M85" s="1">
-        <f>HEX2DEC(L85)</f>
+        <f t="shared" si="3"/>
         <v>77</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.25">
@@ -12091,16 +12091,16 @@
         <v>336</v>
       </c>
       <c r="C86" s="21" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F86" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>54</v>
       </c>
       <c r="G86" s="9">
@@ -12110,20 +12110,20 @@
         <v>336</v>
       </c>
       <c r="I86" s="6" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="L86" s="24" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="M86" s="1">
-        <f>HEX2DEC(L86)</f>
+        <f t="shared" si="3"/>
         <v>78</v>
       </c>
       <c r="N86" s="1" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.25">
@@ -12131,16 +12131,16 @@
         <v>340</v>
       </c>
       <c r="C87" s="21" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F87" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>55</v>
       </c>
       <c r="G87" s="9">
@@ -12150,20 +12150,20 @@
         <v>340</v>
       </c>
       <c r="I87" s="6" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="K87" s="1" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="L87" s="24" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="M87" s="1">
-        <f>HEX2DEC(L87)</f>
+        <f t="shared" si="3"/>
         <v>79</v>
       </c>
       <c r="N87" s="1" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="88" spans="2:14" x14ac:dyDescent="0.25">
@@ -12171,16 +12171,16 @@
         <v>344</v>
       </c>
       <c r="C88" s="23" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F88" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>56</v>
       </c>
       <c r="G88" s="15">
@@ -12190,20 +12190,20 @@
         <v>344</v>
       </c>
       <c r="I88" s="13" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="K88" s="1" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="L88" s="24">
         <v>50</v>
       </c>
       <c r="M88" s="1">
-        <f>HEX2DEC(L88)</f>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.25">
@@ -12211,16 +12211,16 @@
         <v>348</v>
       </c>
       <c r="C89" s="21" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F89" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>57</v>
       </c>
       <c r="G89" s="15">
@@ -12236,16 +12236,16 @@
         <v>352</v>
       </c>
       <c r="C90" s="21" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F90" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>58</v>
       </c>
       <c r="G90" s="15">
@@ -12261,16 +12261,16 @@
         <v>356</v>
       </c>
       <c r="C91" s="21" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F91" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>59</v>
       </c>
       <c r="G91" s="15">
@@ -12286,16 +12286,16 @@
         <v>360</v>
       </c>
       <c r="C92" s="21" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F92" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5A</v>
       </c>
       <c r="G92" s="15">
@@ -12311,16 +12311,16 @@
         <v>364</v>
       </c>
       <c r="C93" s="21" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F93" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5B</v>
       </c>
       <c r="G93" s="15">
@@ -12336,16 +12336,16 @@
         <v>368</v>
       </c>
       <c r="C94" s="21" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F94" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5C</v>
       </c>
       <c r="G94" s="15">
@@ -12361,16 +12361,16 @@
         <v>372</v>
       </c>
       <c r="C95" s="21" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F95" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5D</v>
       </c>
       <c r="G95" s="15">
@@ -12386,16 +12386,16 @@
         <v>376</v>
       </c>
       <c r="C96" s="21" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F96" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5E</v>
       </c>
       <c r="G96" s="15">
@@ -12411,16 +12411,16 @@
         <v>380</v>
       </c>
       <c r="C97" s="21" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F97" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5F</v>
       </c>
       <c r="G97" s="15">
@@ -12436,16 +12436,16 @@
         <v>384</v>
       </c>
       <c r="C98" s="21" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F98" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>60</v>
       </c>
       <c r="G98" s="15">
@@ -12461,16 +12461,16 @@
         <v>388</v>
       </c>
       <c r="C99" s="21" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F99" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>61</v>
       </c>
       <c r="G99" s="9">
@@ -12480,7 +12480,7 @@
         <v>388</v>
       </c>
       <c r="I99" s="6" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="100" spans="2:14" x14ac:dyDescent="0.25">
@@ -12488,16 +12488,16 @@
         <v>392</v>
       </c>
       <c r="C100" s="21" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F100" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>62</v>
       </c>
       <c r="G100" s="9">
@@ -12507,7 +12507,7 @@
         <v>392</v>
       </c>
       <c r="I100" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="101" spans="2:14" x14ac:dyDescent="0.25">
@@ -12515,16 +12515,16 @@
         <v>396</v>
       </c>
       <c r="C101" s="21" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F101" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>63</v>
       </c>
       <c r="G101" s="9">
@@ -12534,7 +12534,7 @@
         <v>396</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="102" spans="2:14" x14ac:dyDescent="0.25">
@@ -12542,16 +12542,16 @@
         <v>400</v>
       </c>
       <c r="C102" s="21" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F102" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>64</v>
       </c>
       <c r="G102" s="9">
@@ -12561,7 +12561,7 @@
         <v>400</v>
       </c>
       <c r="I102" s="6" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="103" spans="2:14" x14ac:dyDescent="0.25">
@@ -12569,16 +12569,16 @@
         <v>404</v>
       </c>
       <c r="C103" s="21" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F103" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>65</v>
       </c>
       <c r="G103" s="9">
@@ -12588,7 +12588,7 @@
         <v>404</v>
       </c>
       <c r="I103" s="6" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="104" spans="2:14" x14ac:dyDescent="0.25">
@@ -12596,16 +12596,16 @@
         <v>408</v>
       </c>
       <c r="C104" s="21" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F104" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>66</v>
       </c>
       <c r="G104" s="9">
@@ -12615,16 +12615,16 @@
         <v>408</v>
       </c>
       <c r="I104" s="6" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="K104" s="1" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="L104" s="24">
         <v>51</v>
       </c>
       <c r="M104" s="1">
-        <f>HEX2DEC(L104)</f>
+        <f t="shared" ref="M104:M109" si="5">HEX2DEC(L104)</f>
         <v>81</v>
       </c>
       <c r="N104" s="1">
@@ -12636,16 +12636,16 @@
         <v>412</v>
       </c>
       <c r="C105" s="21" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F105" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>67</v>
       </c>
       <c r="G105" s="9">
@@ -12655,20 +12655,20 @@
         <v>412</v>
       </c>
       <c r="I105" s="6" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
       <c r="K105" s="1" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="L105" s="24">
         <v>52</v>
       </c>
       <c r="M105" s="1">
-        <f>HEX2DEC(L105)</f>
+        <f t="shared" si="5"/>
         <v>82</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="106" spans="2:14" x14ac:dyDescent="0.25">
@@ -12676,16 +12676,16 @@
         <v>416</v>
       </c>
       <c r="C106" s="21" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F106" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>68</v>
       </c>
       <c r="G106" s="9">
@@ -12695,20 +12695,20 @@
         <v>416</v>
       </c>
       <c r="I106" s="6" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="K106" s="1" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
       <c r="L106" s="24">
         <v>53</v>
       </c>
       <c r="M106" s="1">
-        <f>HEX2DEC(L106)</f>
+        <f t="shared" si="5"/>
         <v>83</v>
       </c>
       <c r="N106" s="1" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="107" spans="2:14" x14ac:dyDescent="0.25">
@@ -12716,16 +12716,16 @@
         <v>420</v>
       </c>
       <c r="C107" s="21" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="D107" s="6" t="s">
+        <v>1222</v>
+      </c>
+      <c r="E107" s="1" t="s">
         <v>1224</v>
       </c>
-      <c r="E107" s="1" t="s">
-        <v>1226</v>
-      </c>
       <c r="F107" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>69</v>
       </c>
       <c r="G107" s="9">
@@ -12735,20 +12735,20 @@
         <v>420</v>
       </c>
       <c r="I107" s="6" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="K107" s="1" t="s">
-        <v>1216</v>
+        <v>1214</v>
       </c>
       <c r="L107" s="24">
         <v>54</v>
       </c>
       <c r="M107" s="1">
-        <f>HEX2DEC(L107)</f>
+        <f t="shared" si="5"/>
         <v>84</v>
       </c>
       <c r="N107" s="1" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="108" spans="2:14" x14ac:dyDescent="0.25">
@@ -12756,16 +12756,16 @@
         <v>424</v>
       </c>
       <c r="C108" s="21" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F108" s="12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6A</v>
       </c>
       <c r="G108" s="9">
@@ -12775,20 +12775,20 @@
         <v>424</v>
       </c>
       <c r="I108" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="K108" s="1" t="s">
-        <v>1217</v>
+        <v>1215</v>
       </c>
       <c r="L108" s="24">
         <v>55</v>
       </c>
       <c r="M108" s="1">
-        <f>HEX2DEC(L108)</f>
+        <f t="shared" si="5"/>
         <v>85</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="109" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -12796,16 +12796,16 @@
         <v>428</v>
       </c>
       <c r="C109" s="23" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="D109" s="26" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
       <c r="F109" s="25" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6B</v>
       </c>
       <c r="G109" s="28">
@@ -12815,21 +12815,21 @@
         <v>428</v>
       </c>
       <c r="I109" s="26" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="J109" s="16"/>
       <c r="K109" s="16" t="s">
-        <v>1218</v>
+        <v>1216</v>
       </c>
       <c r="L109" s="27">
         <v>56</v>
       </c>
       <c r="M109" s="16">
-        <f>HEX2DEC(L109)</f>
+        <f t="shared" si="5"/>
         <v>86</v>
       </c>
       <c r="N109" s="16" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
   </sheetData>

</xml_diff>